<commit_message>
updates metadata with correct units
</commit_message>
<xml_diff>
--- a/data-raw/metadata/clear_redd_metadata.xlsx
+++ b/data-raw/metadata/clear_redd_metadata.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Badhia\Documents\git\jpe-clear-adult-edi\data-raw\metadata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB237A36-D57B-4685-9DD7-3E4CCF318FBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8860A6BB-B97C-41EB-A717-57754C737CCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6740" yWindow="420" windowWidth="19200" windowHeight="11170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5310" yWindow="1820" windowWidth="19200" windowHeight="11170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="attribute" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="63">
   <si>
     <t xml:space="preserve">attribute_name </t>
   </si>
@@ -140,9 +140,6 @@
   </si>
   <si>
     <t>natural</t>
-  </si>
-  <si>
-    <t>meter</t>
   </si>
   <si>
     <t>feetPerSecond</t>
@@ -619,7 +616,7 @@
         <v>20</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>16</v>
@@ -642,7 +639,7 @@
         <v>35</v>
       </c>
       <c r="M2" s="9" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="N2" s="7"/>
       <c r="O2" s="7"/>
@@ -663,7 +660,7 @@
         <v>27</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>22</v>
@@ -701,7 +698,7 @@
         <v>24</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>25</v>
@@ -736,10 +733,10 @@
     </row>
     <row r="5" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>22</v>
@@ -825,7 +822,7 @@
         <v>34</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C7" s="7" t="s">
         <v>22</v>
@@ -850,7 +847,7 @@
         <v>28</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>22</v>
@@ -888,7 +885,7 @@
         <v>29</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>14</v>
@@ -903,7 +900,7 @@
         <v>14</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>38</v>
+        <v>57</v>
       </c>
       <c r="H9" s="6" t="s">
         <v>36</v>
@@ -936,7 +933,7 @@
         <v>30</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>14</v>
@@ -951,7 +948,7 @@
         <v>14</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>38</v>
+        <v>57</v>
       </c>
       <c r="H10" s="6" t="s">
         <v>36</v>
@@ -981,10 +978,10 @@
     </row>
     <row r="11" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>14</v>
@@ -999,7 +996,7 @@
         <v>14</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H11" s="6" t="s">
         <v>36</v>
@@ -1029,10 +1026,10 @@
     </row>
     <row r="12" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>14</v>
@@ -1047,7 +1044,7 @@
         <v>14</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H12" s="6" t="s">
         <v>36</v>
@@ -1077,10 +1074,10 @@
     </row>
     <row r="13" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>14</v>
@@ -1095,7 +1092,7 @@
         <v>14</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H13" s="6" t="s">
         <v>36</v>
@@ -1125,10 +1122,10 @@
     </row>
     <row r="14" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>22</v>
@@ -1163,10 +1160,10 @@
     </row>
     <row r="15" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C15" s="4" t="s">
         <v>22</v>
@@ -1201,10 +1198,10 @@
     </row>
     <row r="16" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>22</v>
@@ -1242,7 +1239,7 @@
         <v>31</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C17" s="4" t="s">
         <v>14</v>
@@ -1257,7 +1254,7 @@
         <v>14</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H17" s="6" t="s">
         <v>36</v>

</xml_diff>

<commit_message>
updates survey reaches on data and metadata
</commit_message>
<xml_diff>
--- a/data-raw/metadata/clear_redd_metadata.xlsx
+++ b/data-raw/metadata/clear_redd_metadata.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Badhia\Documents\git\jpe-clear-adult-edi\data-raw\metadata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8860A6BB-B97C-41EB-A717-57754C737CCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F01A483E-8745-4514-8F7C-F26D1167129A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5310" yWindow="1820" windowWidth="19200" windowHeight="11170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3700" yWindow="1040" windowWidth="19200" windowHeight="11170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="attribute" sheetId="1" r:id="rId1"/>
@@ -154,9 +154,6 @@
     <t>Unique redd ID assigned to the redd being sampled. One redd may have been observed multiple times, resulting in multiple rows for one redd ID.</t>
   </si>
   <si>
-    <t>Survey reach. Levels =c("R1", "R2", "R4", "R3", "R5")</t>
-  </si>
-  <si>
     <t>fish_on_redd</t>
   </si>
   <si>
@@ -218,6 +215,9 @@
   </si>
   <si>
     <t>2024-10-25</t>
+  </si>
+  <si>
+    <t>Survey reach. Levels =c("R1", "R2", "R4", "R3", "R5", "R5A", "R5B", , "R5C")</t>
   </si>
 </sst>
 </file>
@@ -639,7 +639,7 @@
         <v>35</v>
       </c>
       <c r="M2" s="9" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="N2" s="7"/>
       <c r="O2" s="7"/>
@@ -698,7 +698,7 @@
         <v>24</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>42</v>
+        <v>62</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>25</v>
@@ -733,10 +733,10 @@
     </row>
     <row r="5" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>22</v>
@@ -822,7 +822,7 @@
         <v>34</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C7" s="7" t="s">
         <v>22</v>
@@ -847,7 +847,7 @@
         <v>28</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>22</v>
@@ -885,7 +885,7 @@
         <v>29</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>14</v>
@@ -900,7 +900,7 @@
         <v>14</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="H9" s="6" t="s">
         <v>36</v>
@@ -933,7 +933,7 @@
         <v>30</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>14</v>
@@ -948,7 +948,7 @@
         <v>14</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="H10" s="6" t="s">
         <v>36</v>
@@ -978,10 +978,10 @@
     </row>
     <row r="11" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>14</v>
@@ -996,7 +996,7 @@
         <v>14</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="H11" s="6" t="s">
         <v>36</v>
@@ -1026,10 +1026,10 @@
     </row>
     <row r="12" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>14</v>
@@ -1044,7 +1044,7 @@
         <v>14</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="H12" s="6" t="s">
         <v>36</v>
@@ -1074,10 +1074,10 @@
     </row>
     <row r="13" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>14</v>
@@ -1092,7 +1092,7 @@
         <v>14</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="H13" s="6" t="s">
         <v>36</v>
@@ -1122,10 +1122,10 @@
     </row>
     <row r="14" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>22</v>
@@ -1160,10 +1160,10 @@
     </row>
     <row r="15" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C15" s="4" t="s">
         <v>22</v>
@@ -1198,10 +1198,10 @@
     </row>
     <row r="16" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>22</v>

</xml_diff>